<commit_message>
IP valuation: the full 10-K notes add booked reserves; $1.81 a share in all
Reading Notes 10-21 added what a century of mills leaves behind: $270M of environmental
reserves and $103M of asbestos claims net of insurance (after tax), and the $48M IP has
booked for its Brazil tax guarantee to Sylvamo. Debt-like items $957M after tax; DCF
$40.25 -> $38.44; P(value > $32) 63%; the odds the price implies 44%. Pension and lease
inputs now cite Notes 19 and 10 directly. The thesis log's v2 entry says it was revised
the same day and why. The LinkedIn post and caption end with 'I like to build cool sh*t.'

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHTBB4SHCY7nxQ7qSN69vP
</commit_message>
<xml_diff>
--- a/models/ip-valuation/IP_valuation_model.xlsx
+++ b/models/ip-valuation/IP_valuation_model.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="516">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="522">
   <si>
     <t xml:space="preserve">A corrugator engineer values International Paper — model notes</t>
   </si>
@@ -296,7 +296,7 @@
     <t xml:space="preserve">DCF rows: cost of equity = risk-free + β × ERP; after-tax cost of debt = kd × (1 − t); WACC = weights × each. ≈ 7.4%.</t>
   </si>
   <si>
-    <t xml:space="preserve">The hurdle rate. A dollar of cash flow three years out is worth 1/(1.074)^3 ≈ 81¢ today. Raising WACC 1 point knocks ~13% off the value; it is the most-argued number in finance.</t>
+    <t xml:space="preserve">The hurdle rate. A dollar of cash flow three years out is worth 1/(1.074)^3 ≈ 81¢ today. Raising WACC 1 point knocks ~14% off the value; it is the most-argued number in finance.</t>
   </si>
   <si>
     <t xml:space="preserve">Risk-free rate</t>
@@ -413,7 +413,7 @@
     <t xml:space="preserve">Debt minus cash. Plus 'debt-like' items (pension deficits, leases) when material.</t>
   </si>
   <si>
-    <t xml:space="preserve">Inputs: $9,217M − $726M = $8,491M. The 10-K's debt-like items ($626M after tax: pension deficits, retiree medical, the 2027 timber tax net of the notes) come off the equity value, not the WACC weights.</t>
+    <t xml:space="preserve">Inputs: $9,217M − $726M = $8,491M. The 10-K's debt-like items ($957M after tax: pension deficits, retiree medical, the 2027 timber tax net of the notes) come off the equity value, not the WACC weights.</t>
   </si>
   <si>
     <t xml:space="preserve">What the equity holder owes before owning anything. $8.5B against $17B of market cap is a real amount.</t>
@@ -449,7 +449,7 @@
     <t xml:space="preserve">Value each segment at its own multiple, add them, subtract net debt. Used when the parts could be separated or sold.</t>
   </si>
   <si>
-    <t xml:space="preserve">Comps_SOTP: NA 2028E × 9.0× + EMEA × 6.5× − debt − separation costs ≈ $41/share; plus the EMEA multiple at which SOTP = $32.</t>
+    <t xml:space="preserve">Comps_SOTP: NA 2028E × 9.0× + EMEA × 6.5× − debt − separation costs ≈ $40/share; plus the EMEA multiple at which SOTP = $32.</t>
   </si>
   <si>
     <t xml:space="preserve">Live question since Oct 15: DS Smith is for sale or spin. If a buyer pays more than the breakeven multiple, the market is underpricing the sum.</t>
@@ -491,7 +491,7 @@
     <t xml:space="preserve">montecarlo.py: 20,000 runs, same chain as the Scenarios sheet.</t>
   </si>
   <si>
-    <t xml:space="preserve">The point estimate ($39) becomes P(value &gt; $32) = 63% with a 10th percentile of $16. A bet needs the second form.</t>
+    <t xml:space="preserve">The point estimate ($38) becomes P(value &gt; $32) = 62% with a 10th percentile of $16. A bet needs the second form.</t>
   </si>
   <si>
     <t xml:space="preserve">Regime / correlation</t>
@@ -524,7 +524,7 @@
     <t xml:space="preserve">Mean of the outcomes; the middle outcome; the value below which 10% (90%) of outcomes fall.</t>
   </si>
   <si>
-    <t xml:space="preserve">mc.json: mean $37, median $38, 10th $16, 90th $55.</t>
+    <t xml:space="preserve">mc.json: mean $36, median $37, 10th $16, 90th $54.</t>
   </si>
   <si>
     <t xml:space="preserve">The 10th percentile is the number to size against, not the mean.</t>
@@ -536,7 +536,7 @@
     <t xml:space="preserve">The P(down-cycle) at which the expected value equals the price.</t>
   </si>
   <si>
-    <t xml:space="preserve">mc_pdown.json: ≈ 48%.</t>
+    <t xml:space="preserve">mc_pdown.json: ≈ 46%.</t>
   </si>
   <si>
     <t xml:space="preserve">What the market is 'saying' at $32: a coin flip on the cycle. Your edge is whether you can call it better than a coin.</t>
@@ -548,7 +548,7 @@
     <t xml:space="preserve">The fraction of capital that maximizes long-run growth given a known payoff distribution: f* = argmax E[log(1 + f·r)].</t>
   </si>
   <si>
-    <t xml:space="preserve">montecarlo.py: numeric Kelly ≈ 0.68; half-Kelly 0.34.</t>
+    <t xml:space="preserve">montecarlo.py: numeric Kelly ≈ 0.59; half-Kelly 0.29.</t>
   </si>
   <si>
     <t xml:space="preserve">Assumes you KNOW the distribution. You don't; you assigned the 30%. Treat it as a ceiling, then divide by the number of things you could be wrong about. For one cyclical stock: small.</t>
@@ -560,7 +560,7 @@
     <t xml:space="preserve">Buy below your estimate of value by enough to be wrong and still be fine.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mid-case $39 vs $32 ≈ 18% — modest for a cyclical with uncovered dividend; the Monte Carlo's 10th percentile ($16) is the honest version.</t>
+    <t xml:space="preserve">Mid-case $38 vs $32 ≈ 17% — modest for a cyclical with uncovered dividend; the Monte Carlo's 10th percentile ($16) is the honest version.</t>
   </si>
   <si>
     <t xml:space="preserve">The same instinct as leaving a half-inch of trim rather than running the chute at 7.0.</t>
@@ -683,37 +683,55 @@
     <t xml:space="preserve">Pensions, all plans: assets above obligations (the filing's net)</t>
   </si>
   <si>
-    <t xml:space="preserve">10-K MD&amp;A: 'the projected benefit obligation ... was approximately $144 million lower than the fair value of plan assets.' (Risk Factors says $148M; the plan table gives 144.)</t>
+    <t xml:space="preserve">10-K MD&amp;A: 'the projected benefit obligation ... was approximately $144 million lower than the fair value of plan assets.' Note 19: U.S. plans +$148M, non-U.S. −$4M.</t>
   </si>
   <si>
     <t xml:space="preserve">Pension plans in surplus, total (not counted by default)</t>
   </si>
   <si>
-    <t xml:space="preserve">10-K balance sheet: Overfunded Pension Plan Assets $486M.</t>
+    <t xml:space="preserve">10-K Note 19, noncurrent assets: U.S. $367M + non-U.S. $119M = $486M (balance sheet: Overfunded Pension Plan Assets $486M).</t>
   </si>
   <si>
     <t xml:space="preserve">Pension plans in deficit, total (counted, after tax)</t>
   </si>
   <si>
-    <t xml:space="preserve">Surplus plans $486M less the $144M net = $342M owed by plans in deficit (balance sheet: Underfunded Pension Benefit Obligations $316M long-term, the rest current).</t>
+    <t xml:space="preserve">10-K Note 19, liabilities: U.S. $21M current + $198M noncurrent, non-U.S. $5M current + $118M noncurrent = $342M (balance sheet: Underfunded Pension Benefit Obligations $316M long-term).</t>
   </si>
   <si>
     <t xml:space="preserve">Retiree medical and postemployment benefits (counted, after tax)</t>
   </si>
   <si>
-    <t xml:space="preserve">10-K balance sheet: Postretirement and Postemployment Benefit Obligation $133M (long-term).</t>
+    <t xml:space="preserve">10-K balance sheet: Postretirement and Postemployment Benefit Obligation $133M. Note 19 calls the other postretirement plans 'not considered material' and gives no table.</t>
   </si>
   <si>
     <t xml:space="preserve">Operating lease liabilities (not counted: the lease cost is already inside EBITDA)</t>
   </si>
   <si>
-    <t xml:space="preserve">Dec 31, 2025: $221M current + $486M long-term (Q1 2026 10-Q lease table, December 31, 2025 column; the 10-K balance sheet shows Long-Term Lease Obligations $486M and Right of Use Assets $697M). Under U.S. GAAP operating lease cost is an operating expense, so EBITDA is after rent; adding the liability too would count it twice.</t>
+    <t xml:space="preserve">10-K Note 10: operating lease liabilities $221M current (other current liabilities) + $486M noncurrent (long-term lease obligations); 2025 operating lease cost $258M. Under U.S. GAAP operating lease cost is an operating expense, so EBITDA is after rent; adding the liability too would count it twice.</t>
   </si>
   <si>
     <t xml:space="preserve">Finance lease liabilities (not counted again: already inside gross debt)</t>
   </si>
   <si>
-    <t xml:space="preserve">Dec 31, 2025: $17M in current maturities of debt + $54M in long-term debt (Q1 2026 10-Q lease table, December 31, 2025 column); the 10-K's debt maturities 'include financing lease obligations'.</t>
+    <t xml:space="preserve">10-K Note 10: finance lease liabilities $17M in notes payable and current maturities of long-term debt + $54M in long-term debt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Environmental remediation reserves, old mill sites (counted, after tax)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-K Note 14: 'International Paper's estimated probable liability for these environmental matters, totaled approximately $270 million' at Dec 31, 2025 (Cass Lake, Kalamazoo River, San Jacinto, Versailles Pond among them). Remediation is a special item, outside adjusted EBITDA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asbestos claims, net of insurance (counted, after tax)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-K Note 14: 'total recorded liability with respect to pending and future asbestos-related claims was $103 million ... net of insurance recoveries'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brazil tax guarantee to Sylvamo, already booked (counted in full)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-K Note 14: 'The initial fair value estimate and recorded liability as of December 31, 2021 was $48 million and remains this amount at December 31, 2025.'</t>
   </si>
   <si>
     <t xml:space="preserve">Deferred tax on the Temple-Inland timber notes, due 2027 (counted)</t>
@@ -725,7 +743,7 @@
     <t xml:space="preserve">Timber notes held by the special purpose entities (counted, net of the loans)</t>
   </si>
   <si>
-    <t xml:space="preserve">10-K balance sheet: Long-Term Financial Assets of Variable Interest Entities $2,349M.</t>
+    <t xml:space="preserve">10-K balance sheet: Long-Term Financial Assets of Variable Interest Entities $2,349M. Note 15: $2.4B face, due 2027, backed by letters of credit from three banks.</t>
   </si>
   <si>
     <t xml:space="preserve">Nonrecourse loans against those notes</t>
@@ -746,7 +764,7 @@
     <t xml:space="preserve">10-K contractual obligations footnote: 'approximately $344 million of unrecognized tax benefits'.</t>
   </si>
   <si>
-    <t xml:space="preserve">Brazil tax matter via the Sylvamo agreement, IP's share (not counted: contingent, not booked)</t>
+    <t xml:space="preserve">Brazil tax matter via the Sylvamo agreement, IP's potential share (counted only the $48M booked)</t>
   </si>
   <si>
     <t xml:space="preserve">10-K Risk Factors: 'our potential liability for such assessments would currently be approximately $274 million' (assessments total about $394M, 2007–2015 tax years).</t>
@@ -767,7 +785,7 @@
     <t xml:space="preserve">DERIVED</t>
   </si>
   <si>
-    <t xml:space="preserve">Pension deficits + retiree medical, after tax; minus the surplus if counted; plus the 2027 timber tax; minus the equity in the timber structure (notes less loans). Operating leases excluded.</t>
+    <t xml:space="preserve">Pension deficits, retiree medical, environmental and asbestos reserves, after tax; the booked Brazil guarantee; the 2027 timber tax less the equity in the timber structure (notes less loans); minus the pension surplus only if counted. Operating leases excluded.</t>
   </si>
   <si>
     <t xml:space="preserve">Latest reported and guided financials</t>
@@ -2969,7 +2987,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E92"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -3311,7 +3329,7 @@
         <v>229</v>
       </c>
       <c r="B29" s="17" t="n">
-        <v>487</v>
+        <v>270</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>191</v>
@@ -3325,7 +3343,7 @@
         <v>231</v>
       </c>
       <c r="B30" s="17" t="n">
-        <v>2349</v>
+        <v>103</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>191</v>
@@ -3339,7 +3357,7 @@
         <v>233</v>
       </c>
       <c r="B31" s="17" t="n">
-        <v>2127</v>
+        <v>48</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>191</v>
@@ -3353,7 +3371,7 @@
         <v>235</v>
       </c>
       <c r="B32" s="17" t="n">
-        <v>2584</v>
+        <v>487</v>
       </c>
       <c r="C32" s="7" t="s">
         <v>191</v>
@@ -3367,7 +3385,7 @@
         <v>237</v>
       </c>
       <c r="B33" s="17" t="n">
-        <v>344</v>
+        <v>2349</v>
       </c>
       <c r="C33" s="7" t="s">
         <v>191</v>
@@ -3381,7 +3399,7 @@
         <v>239</v>
       </c>
       <c r="B34" s="17" t="n">
-        <v>274</v>
+        <v>2127</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>191</v>
@@ -3394,88 +3412,88 @@
       <c r="A35" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="B35" s="18" t="n">
-        <v>0</v>
+      <c r="B35" s="17" t="n">
+        <v>2584</v>
       </c>
       <c r="C35" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="E35" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="E35" s="7" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="B36" s="17" t="n">
+        <v>344</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="E36" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="B36" s="19" t="n">
-        <f aca="false">(Inputs!$B$25+Inputs!$B$26)*(1-Inputs!$B$75)-Inputs!$B$24*(1-Inputs!$B$75)*Inputs!$B$35+Inputs!$B$29-(Inputs!$B$30-Inputs!$B$31)</f>
-        <v>626</v>
-      </c>
-      <c r="C36" s="7" t="s">
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="E36" s="7" t="s">
+      <c r="B37" s="17" t="n">
+        <v>274</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="E37" s="7" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="B38" s="9"/>
-      <c r="C38" s="9"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
+      <c r="B38" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="B39" s="17" t="n">
-        <v>15000</v>
+        <v>250</v>
+      </c>
+      <c r="B39" s="19" t="n">
+        <f aca="false">(Inputs!$B$25+Inputs!$B$26+Inputs!$B$29+Inputs!$B$30)*(1-Inputs!$B$78)-Inputs!$B$24*(1-Inputs!$B$78)*Inputs!$B$38+Inputs!$B$31+Inputs!$B$32-(Inputs!$B$33-Inputs!$B$34)</f>
+        <v>957.48</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>191</v>
+        <v>251</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="12" t="s">
-        <v>250</v>
-      </c>
-      <c r="B40" s="17" t="n">
-        <v>8500</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="E40" s="7" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="12" t="s">
-        <v>252</v>
-      </c>
-      <c r="B41" s="17" t="n">
-        <v>2300</v>
-      </c>
-      <c r="C41" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="E41" s="7" t="s">
+      <c r="A41" s="8" t="s">
         <v>253</v>
       </c>
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
         <v>254</v>
       </c>
       <c r="B42" s="17" t="n">
-        <v>800</v>
+        <v>15000</v>
       </c>
       <c r="C42" s="7" t="s">
         <v>191</v>
@@ -3489,7 +3507,7 @@
         <v>256</v>
       </c>
       <c r="B43" s="17" t="n">
-        <v>-159</v>
+        <v>8500</v>
       </c>
       <c r="C43" s="7" t="s">
         <v>191</v>
@@ -3503,7 +3521,7 @@
         <v>258</v>
       </c>
       <c r="B44" s="17" t="n">
-        <v>11975</v>
+        <v>2300</v>
       </c>
       <c r="C44" s="7" t="s">
         <v>191</v>
@@ -3517,7 +3535,7 @@
         <v>260</v>
       </c>
       <c r="B45" s="17" t="n">
-        <v>1264</v>
+        <v>800</v>
       </c>
       <c r="C45" s="7" t="s">
         <v>191</v>
@@ -3531,7 +3549,7 @@
         <v>262</v>
       </c>
       <c r="B46" s="17" t="n">
-        <v>1050</v>
+        <v>-159</v>
       </c>
       <c r="C46" s="7" t="s">
         <v>191</v>
@@ -3545,52 +3563,52 @@
         <v>264</v>
       </c>
       <c r="B47" s="17" t="n">
-        <v>3200</v>
+        <v>11975</v>
       </c>
       <c r="C47" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="E47" s="7" t="s">
         <v>265</v>
-      </c>
-      <c r="E47" s="7" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="B48" s="17" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="E48" s="7" t="s">
         <v>267</v>
-      </c>
-      <c r="B48" s="17" t="n">
-        <v>3400</v>
-      </c>
-      <c r="C48" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="E48" s="7" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="B49" s="17" t="n">
+        <v>1050</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="E49" s="7" t="s">
         <v>269</v>
-      </c>
-      <c r="B49" s="17" t="n">
-        <v>3500</v>
-      </c>
-      <c r="C49" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="E49" s="7" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="B50" s="17" t="n">
+        <v>3200</v>
+      </c>
+      <c r="C50" s="7" t="s">
         <v>271</v>
-      </c>
-      <c r="B50" s="17" t="n">
-        <v>3700</v>
-      </c>
-      <c r="C50" s="7" t="s">
-        <v>265</v>
       </c>
       <c r="E50" s="7" t="s">
         <v>272</v>
@@ -3601,10 +3619,10 @@
         <v>273</v>
       </c>
       <c r="B51" s="17" t="n">
-        <v>2425</v>
+        <v>3400</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="E51" s="7" t="s">
         <v>274</v>
@@ -3615,10 +3633,10 @@
         <v>275</v>
       </c>
       <c r="B52" s="17" t="n">
-        <v>950</v>
+        <v>3500</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="E52" s="7" t="s">
         <v>276</v>
@@ -3629,10 +3647,10 @@
         <v>277</v>
       </c>
       <c r="B53" s="17" t="n">
-        <v>1965</v>
+        <v>3700</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="E53" s="7" t="s">
         <v>278</v>
@@ -3643,10 +3661,10 @@
         <v>279</v>
       </c>
       <c r="B54" s="17" t="n">
-        <v>370</v>
+        <v>2425</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="E54" s="7" t="s">
         <v>280</v>
@@ -3657,10 +3675,10 @@
         <v>281</v>
       </c>
       <c r="B55" s="17" t="n">
-        <v>400</v>
+        <v>950</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="E55" s="7" t="s">
         <v>282</v>
@@ -3670,76 +3688,76 @@
       <c r="A56" s="12" t="s">
         <v>283</v>
       </c>
-      <c r="B56" s="20" t="n">
-        <v>250</v>
+      <c r="B56" s="17" t="n">
+        <v>1965</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="E56" s="7" t="s">
         <v>284</v>
       </c>
     </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="B57" s="17" t="n">
+        <v>370</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>286</v>
+      </c>
+    </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="8" t="s">
-        <v>285</v>
-      </c>
-      <c r="B58" s="9"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9"/>
+      <c r="A58" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="B58" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="E58" s="7" t="s">
+        <v>288</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="s">
-        <v>286</v>
-      </c>
-      <c r="B59" s="17" t="n">
-        <v>170</v>
+        <v>289</v>
+      </c>
+      <c r="B59" s="20" t="n">
+        <v>250</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>188</v>
+        <v>248</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="12" t="s">
-        <v>288</v>
-      </c>
-      <c r="B60" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="C60" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="E60" s="7" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="12" t="s">
-        <v>290</v>
-      </c>
-      <c r="B61" s="17" t="n">
-        <v>175</v>
-      </c>
-      <c r="C61" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="E61" s="7" t="s">
+      <c r="A61" s="8" t="s">
         <v>291</v>
       </c>
+      <c r="B61" s="9"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="9"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="12" t="s">
         <v>292</v>
       </c>
-      <c r="B62" s="21" t="n">
-        <v>0.5</v>
+      <c r="B62" s="17" t="n">
+        <v>170</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>242</v>
+        <v>188</v>
       </c>
       <c r="E62" s="7" t="s">
         <v>293</v>
@@ -3749,11 +3767,11 @@
       <c r="A63" s="12" t="s">
         <v>294</v>
       </c>
-      <c r="B63" s="21" t="n">
-        <v>0.01</v>
+      <c r="B63" s="17" t="n">
+        <v>9</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="E63" s="7" t="s">
         <v>295</v>
@@ -3763,11 +3781,11 @@
       <c r="A64" s="12" t="s">
         <v>296</v>
       </c>
-      <c r="B64" s="21" t="n">
-        <v>0.3</v>
+      <c r="B64" s="17" t="n">
+        <v>175</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="E64" s="7" t="s">
         <v>297</v>
@@ -3777,11 +3795,11 @@
       <c r="A65" s="12" t="s">
         <v>298</v>
       </c>
-      <c r="B65" s="20" t="n">
-        <v>300</v>
+      <c r="B65" s="21" t="n">
+        <v>0.5</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E65" s="7" t="s">
         <v>299</v>
@@ -3791,11 +3809,11 @@
       <c r="A66" s="12" t="s">
         <v>300</v>
       </c>
-      <c r="B66" s="20" t="n">
-        <v>250</v>
+      <c r="B66" s="21" t="n">
+        <v>0.01</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E66" s="7" t="s">
         <v>301</v>
@@ -3805,11 +3823,11 @@
       <c r="A67" s="12" t="s">
         <v>302</v>
       </c>
-      <c r="B67" s="20" t="n">
-        <v>150</v>
+      <c r="B67" s="21" t="n">
+        <v>0.3</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E67" s="7" t="s">
         <v>303</v>
@@ -3819,11 +3837,11 @@
       <c r="A68" s="12" t="s">
         <v>304</v>
       </c>
-      <c r="B68" s="21" t="n">
-        <v>0.17</v>
+      <c r="B68" s="20" t="n">
+        <v>300</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E68" s="7" t="s">
         <v>305</v>
@@ -3833,11 +3851,11 @@
       <c r="A69" s="12" t="s">
         <v>306</v>
       </c>
-      <c r="B69" s="21" t="n">
-        <v>0.11</v>
+      <c r="B69" s="20" t="n">
+        <v>250</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E69" s="7" t="s">
         <v>307</v>
@@ -3847,11 +3865,11 @@
       <c r="A70" s="12" t="s">
         <v>308</v>
       </c>
-      <c r="B70" s="21" t="n">
-        <v>0.025</v>
+      <c r="B70" s="20" t="n">
+        <v>150</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E70" s="7" t="s">
         <v>309</v>
@@ -3861,11 +3879,11 @@
       <c r="A71" s="12" t="s">
         <v>310</v>
       </c>
-      <c r="B71" s="20" t="n">
-        <v>1900</v>
+      <c r="B71" s="21" t="n">
+        <v>0.17</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E71" s="7" t="s">
         <v>311</v>
@@ -3876,10 +3894,10 @@
         <v>312</v>
       </c>
       <c r="B72" s="21" t="n">
-        <v>0.065</v>
+        <v>0.11</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E72" s="7" t="s">
         <v>313</v>
@@ -3890,10 +3908,10 @@
         <v>314</v>
       </c>
       <c r="B73" s="21" t="n">
-        <v>0.08</v>
+        <v>0.025</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E73" s="7" t="s">
         <v>315</v>
@@ -3903,11 +3921,11 @@
       <c r="A74" s="12" t="s">
         <v>316</v>
       </c>
-      <c r="B74" s="21" t="n">
-        <v>0.1</v>
+      <c r="B74" s="20" t="n">
+        <v>1900</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E74" s="7" t="s">
         <v>317</v>
@@ -3918,72 +3936,72 @@
         <v>318</v>
       </c>
       <c r="B75" s="21" t="n">
-        <v>0.24</v>
+        <v>0.065</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E75" s="7" t="s">
         <v>319</v>
       </c>
     </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="12" t="s">
+        <v>320</v>
+      </c>
+      <c r="B76" s="21" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="E76" s="7" t="s">
+        <v>321</v>
+      </c>
+    </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="8" t="s">
-        <v>320</v>
-      </c>
-      <c r="B77" s="9"/>
-      <c r="C77" s="9"/>
-      <c r="D77" s="9"/>
-      <c r="E77" s="9"/>
+      <c r="A77" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="B77" s="21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C77" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="E77" s="7" t="s">
+        <v>323</v>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B78" s="21" t="n">
-        <v>0.04</v>
+        <v>0.24</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>188</v>
+        <v>248</v>
       </c>
       <c r="E78" s="7" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="12" t="s">
-        <v>323</v>
-      </c>
-      <c r="B79" s="22" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C79" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="E79" s="7" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="12" t="s">
-        <v>325</v>
-      </c>
-      <c r="B80" s="21" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="C80" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="E80" s="7" t="s">
+      <c r="A80" s="8" t="s">
         <v>326</v>
       </c>
+      <c r="B80" s="9"/>
+      <c r="C80" s="9"/>
+      <c r="D80" s="9"/>
+      <c r="E80" s="9"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
         <v>327</v>
       </c>
       <c r="B81" s="21" t="n">
-        <v>0.055</v>
+        <v>0.04</v>
       </c>
       <c r="C81" s="7" t="s">
         <v>188</v>
@@ -3996,11 +4014,11 @@
       <c r="A82" s="12" t="s">
         <v>329</v>
       </c>
-      <c r="B82" s="21" t="n">
-        <v>0.02</v>
+      <c r="B82" s="22" t="n">
+        <v>1.1</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E82" s="7" t="s">
         <v>330</v>
@@ -4010,102 +4028,144 @@
       <c r="A83" s="12" t="s">
         <v>331</v>
       </c>
-      <c r="B83" s="23" t="n">
-        <v>8</v>
+      <c r="B83" s="21" t="n">
+        <v>0.045</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E83" s="7" t="s">
         <v>332</v>
       </c>
     </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="B84" s="21" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="C84" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="E84" s="7" t="s">
+        <v>334</v>
+      </c>
+    </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="8" t="s">
-        <v>333</v>
-      </c>
-      <c r="B85" s="9"/>
-      <c r="C85" s="9"/>
-      <c r="D85" s="9"/>
-      <c r="E85" s="9"/>
+      <c r="A85" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="B85" s="21" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C85" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="E85" s="7" t="s">
+        <v>336</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>334</v>
-      </c>
-      <c r="B86" s="24" t="n">
-        <v>12.2</v>
+        <v>337</v>
+      </c>
+      <c r="B86" s="23" t="n">
+        <v>8</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>188</v>
+        <v>248</v>
       </c>
       <c r="E86" s="7" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="12" t="s">
-        <v>336</v>
-      </c>
-      <c r="B87" s="16" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="C87" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="E87" s="7" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="12" t="s">
-        <v>338</v>
-      </c>
-      <c r="B88" s="24" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="C88" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="E88" s="7" t="s">
+      <c r="A88" s="8" t="s">
         <v>339</v>
       </c>
+      <c r="B88" s="9"/>
+      <c r="C88" s="9"/>
+      <c r="D88" s="9"/>
+      <c r="E88" s="9"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="s">
         <v>340</v>
       </c>
-      <c r="B89" s="16" t="n">
-        <v>0.15</v>
+      <c r="B89" s="24" t="n">
+        <v>12.2</v>
       </c>
       <c r="C89" s="7" t="s">
         <v>188</v>
       </c>
       <c r="E89" s="7" t="s">
-        <v>337</v>
+        <v>341</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="12" t="s">
+        <v>342</v>
+      </c>
+      <c r="B90" s="16" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="C90" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="E90" s="7" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="B91" s="9"/>
-      <c r="C91" s="9"/>
-      <c r="D91" s="9"/>
-      <c r="E91" s="9"/>
+      <c r="A91" s="12" t="s">
+        <v>344</v>
+      </c>
+      <c r="B91" s="24" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="C91" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="E91" s="7" t="s">
+        <v>345</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="B92" s="25" t="n">
-        <v>2</v>
+        <v>346</v>
+      </c>
+      <c r="B92" s="16" t="n">
+        <v>0.15</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>242</v>
+        <v>188</v>
       </c>
       <c r="E92" s="7" t="s">
         <v>343</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="B94" s="9"/>
+      <c r="C94" s="9"/>
+      <c r="D94" s="9"/>
+      <c r="E94" s="9"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="12" t="s">
+        <v>348</v>
+      </c>
+      <c r="B95" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C95" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="E95" s="7" t="s">
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -4134,43 +4194,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="E4" s="26" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="F4" s="26" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="G4" s="26" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="B5" s="28"/>
       <c r="C5" s="28"/>
@@ -4182,71 +4242,71 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="B6" s="30" t="n">
-        <f aca="false">Inputs!$B$39</f>
+        <f aca="false">Inputs!$B$42</f>
         <v>15000</v>
       </c>
       <c r="C6" s="31" t="n">
-        <f aca="false">Inputs!$B$44*2*Inputs!$B$39/(Inputs!$B$39+Inputs!$B$40)</f>
+        <f aca="false">Inputs!$B$47*2*Inputs!$B$42/(Inputs!$B$42+Inputs!$B$43)</f>
         <v>15287.2340425532</v>
       </c>
       <c r="D6" s="32" t="n">
-        <f aca="false">C6*(1+Inputs!$B$63)+Inputs!$B$62*Inputs!$B$59*Inputs!$B$60-Inputs!$B$61</f>
+        <f aca="false">C6*(1+Inputs!$B$66)+Inputs!$B$65*Inputs!$B$62*Inputs!$B$63-Inputs!$B$64</f>
         <v>16030.1063829787</v>
       </c>
       <c r="E6" s="32" t="n">
-        <f aca="false">D6*(1+Inputs!$B$70)</f>
+        <f aca="false">D6*(1+Inputs!$B$73)</f>
         <v>16430.8590425532</v>
       </c>
       <c r="F6" s="32" t="n">
-        <f aca="false">E6*(1+Inputs!$B$70)</f>
+        <f aca="false">E6*(1+Inputs!$B$73)</f>
         <v>16841.630518617</v>
       </c>
       <c r="G6" s="32" t="n">
-        <f aca="false">F6*(1+Inputs!$B$70)</f>
+        <f aca="false">F6*(1+Inputs!$B$73)</f>
         <v>17262.6712815824</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="B7" s="30" t="n">
-        <f aca="false">Inputs!$B$40</f>
+        <f aca="false">Inputs!$B$43</f>
         <v>8500</v>
       </c>
       <c r="C7" s="31" t="n">
-        <f aca="false">Inputs!$B$44*2*Inputs!$B$40/(Inputs!$B$39+Inputs!$B$40)</f>
+        <f aca="false">Inputs!$B$47*2*Inputs!$B$43/(Inputs!$B$42+Inputs!$B$43)</f>
         <v>8662.76595744681</v>
       </c>
       <c r="D7" s="31" t="n">
-        <f aca="false">C7*(1+Inputs!$B$70)</f>
+        <f aca="false">C7*(1+Inputs!$B$73)</f>
         <v>8879.33510638298</v>
       </c>
       <c r="E7" s="32" t="n">
-        <f aca="false">D7*(1+Inputs!$B$70)</f>
+        <f aca="false">D7*(1+Inputs!$B$73)</f>
         <v>9101.31848404255</v>
       </c>
       <c r="F7" s="32" t="n">
-        <f aca="false">E7*(1+Inputs!$B$70)</f>
+        <f aca="false">E7*(1+Inputs!$B$73)</f>
         <v>9328.85144614361</v>
       </c>
       <c r="G7" s="32" t="n">
-        <f aca="false">F7*(1+Inputs!$B$70)</f>
+        <f aca="false">F7*(1+Inputs!$B$73)</f>
         <v>9562.0727322972</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="B8" s="33" t="n">
         <f aca="false">B6+B7</f>
@@ -4275,7 +4335,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="B9" s="34"/>
       <c r="C9" s="35" t="n">
@@ -4301,7 +4361,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="B10" s="28"/>
       <c r="C10" s="28"/>
@@ -4313,66 +4373,66 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="B11" s="30" t="n">
-        <f aca="false">Inputs!$B$41</f>
+        <f aca="false">Inputs!$B$44</f>
         <v>2300</v>
       </c>
       <c r="C11" s="30" t="n">
-        <f aca="false">Inputs!$B$51</f>
+        <f aca="false">Inputs!$B$54</f>
         <v>2425</v>
       </c>
       <c r="D11" s="32" t="n">
-        <f aca="false">C11+(Inputs!$B$62*Inputs!$B$59*Inputs!$B$60-Inputs!$B$61)+C6*Inputs!$B$63*Inputs!$B$64+Inputs!$B$65*C6/C8-Inputs!$B$66*C6/C8</f>
+        <f aca="false">C11+(Inputs!$B$65*Inputs!$B$62*Inputs!$B$63-Inputs!$B$64)+C6*Inputs!$B$66*Inputs!$B$67+Inputs!$B$68*C6/C8-Inputs!$B$69*C6/C8</f>
         <v>3092.77659574468</v>
       </c>
       <c r="E11" s="32" t="n">
-        <f aca="false">E6*Inputs!$B$68</f>
+        <f aca="false">E6*Inputs!$B$71</f>
         <v>2793.24603723404</v>
       </c>
       <c r="F11" s="32" t="n">
-        <f aca="false">F6*Inputs!$B$68</f>
+        <f aca="false">F6*Inputs!$B$71</f>
         <v>2863.07718816489</v>
       </c>
       <c r="G11" s="32" t="n">
-        <f aca="false">G6*Inputs!$B$68</f>
+        <f aca="false">G6*Inputs!$B$71</f>
         <v>2934.65411786902</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="B12" s="30" t="n">
-        <f aca="false">Inputs!$B$42</f>
+        <f aca="false">Inputs!$B$45</f>
         <v>800</v>
       </c>
       <c r="C12" s="30" t="n">
-        <f aca="false">Inputs!$B$52</f>
+        <f aca="false">Inputs!$B$55</f>
         <v>950</v>
       </c>
       <c r="D12" s="32" t="n">
-        <f aca="false">C12+Inputs!$B$67+(Inputs!$B$65-Inputs!$B$66)*C7/C8</f>
+        <f aca="false">C12+Inputs!$B$70+(Inputs!$B$68-Inputs!$B$69)*C7/C8</f>
         <v>1118.08510638298</v>
       </c>
       <c r="E12" s="32" t="n">
-        <f aca="false">E7*Inputs!$B$69</f>
+        <f aca="false">E7*Inputs!$B$72</f>
         <v>1001.14503324468</v>
       </c>
       <c r="F12" s="32" t="n">
-        <f aca="false">F7*Inputs!$B$69</f>
+        <f aca="false">F7*Inputs!$B$72</f>
         <v>1026.1736590758</v>
       </c>
       <c r="G12" s="32" t="n">
-        <f aca="false">G7*Inputs!$B$69</f>
+        <f aca="false">G7*Inputs!$B$72</f>
         <v>1051.82800055269</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4383,7 +4443,7 @@
         <v>-100</v>
       </c>
       <c r="C13" s="31" t="n">
-        <f aca="false">(Inputs!$B$47+Inputs!$B$48)/2-Inputs!$B$51-Inputs!$B$52</f>
+        <f aca="false">(Inputs!$B$50+Inputs!$B$51)/2-Inputs!$B$54-Inputs!$B$55</f>
         <v>-75</v>
       </c>
       <c r="D13" s="31" t="n">
@@ -4403,12 +4463,12 @@
         <v>-75</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="B14" s="33" t="n">
         <f aca="false">B11+B12+B13</f>
@@ -4437,7 +4497,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="B15" s="35" t="n">
         <f aca="false">B14/B8</f>
@@ -4466,7 +4526,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="B16" s="35" t="n">
         <f aca="false">B11/B6</f>
@@ -4493,12 +4553,12 @@
         <v>0.17</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="B17" s="35" t="n">
         <f aca="false">B12/B7</f>
@@ -4527,7 +4587,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="27" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="B18" s="28"/>
       <c r="C18" s="28"/>
@@ -4539,39 +4599,39 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="B19" s="31" t="n">
-        <f aca="false">-Inputs!$B$53*0.95</f>
+        <f aca="false">-Inputs!$B$56*0.95</f>
         <v>-1866.75</v>
       </c>
       <c r="C19" s="31" t="n">
-        <f aca="false">-Inputs!$B$53</f>
+        <f aca="false">-Inputs!$B$56</f>
         <v>-1965</v>
       </c>
       <c r="D19" s="31" t="n">
-        <f aca="false">-D8*Inputs!$B$73</f>
+        <f aca="false">-D8*Inputs!$B$76</f>
         <v>-1992.75531914894</v>
       </c>
       <c r="E19" s="31" t="n">
-        <f aca="false">-E8*Inputs!$B$73</f>
+        <f aca="false">-E8*Inputs!$B$76</f>
         <v>-2042.57420212766</v>
       </c>
       <c r="F19" s="31" t="n">
-        <f aca="false">-F8*Inputs!$B$73</f>
+        <f aca="false">-F8*Inputs!$B$76</f>
         <v>-2093.63855718085</v>
       </c>
       <c r="G19" s="31" t="n">
-        <f aca="false">-G8*Inputs!$B$73</f>
+        <f aca="false">-G8*Inputs!$B$76</f>
         <v>-2145.97952111037</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="B20" s="33" t="n">
         <f aca="false">B14+B19</f>
@@ -4600,34 +4660,34 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="B21" s="31" t="n">
-        <f aca="false">-MAX(0,B20)*Inputs!$B$75</f>
+        <f aca="false">-MAX(0,B20)*Inputs!$B$78</f>
         <v>-271.98</v>
       </c>
       <c r="C21" s="31" t="n">
-        <f aca="false">-MAX(0,C20)*Inputs!$B$75</f>
+        <f aca="false">-MAX(0,C20)*Inputs!$B$78</f>
         <v>-320.4</v>
       </c>
       <c r="D21" s="31" t="n">
-        <f aca="false">-MAX(0,D20)*Inputs!$B$75</f>
+        <f aca="false">-MAX(0,D20)*Inputs!$B$78</f>
         <v>-514.345531914894</v>
       </c>
       <c r="E21" s="31" t="n">
-        <f aca="false">-MAX(0,E20)*Inputs!$B$75</f>
+        <f aca="false">-MAX(0,E20)*Inputs!$B$78</f>
         <v>-402.436048404255</v>
       </c>
       <c r="F21" s="31" t="n">
-        <f aca="false">-MAX(0,F20)*Inputs!$B$75</f>
+        <f aca="false">-MAX(0,F20)*Inputs!$B$78</f>
         <v>-412.946949614362</v>
       </c>
       <c r="G21" s="31" t="n">
-        <f aca="false">-MAX(0,G20)*Inputs!$B$75</f>
+        <f aca="false">-MAX(0,G20)*Inputs!$B$78</f>
         <v>-423.720623354721</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4661,7 +4721,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="B23" s="31" t="n">
         <f aca="false">-B19</f>
@@ -4690,72 +4750,72 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="B24" s="31" t="n">
         <v>-2000</v>
       </c>
       <c r="C24" s="31" t="n">
-        <f aca="false">-Inputs!$B$46*2</f>
+        <f aca="false">-Inputs!$B$49*2</f>
         <v>-2100</v>
       </c>
       <c r="D24" s="31" t="n">
-        <f aca="false">-Inputs!$B$71</f>
+        <f aca="false">-Inputs!$B$74</f>
         <v>-1900</v>
       </c>
       <c r="E24" s="31" t="n">
-        <f aca="false">-E8*Inputs!$B$72</f>
+        <f aca="false">-E8*Inputs!$B$75</f>
         <v>-1659.59153922872</v>
       </c>
       <c r="F24" s="31" t="n">
-        <f aca="false">-F8*Inputs!$B$72</f>
+        <f aca="false">-F8*Inputs!$B$75</f>
         <v>-1701.08132770944</v>
       </c>
       <c r="G24" s="31" t="n">
-        <f aca="false">-G8*Inputs!$B$72</f>
+        <f aca="false">-G8*Inputs!$B$75</f>
         <v>-1743.60836090218</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="B25" s="34"/>
       <c r="C25" s="31" t="n">
-        <f aca="false">-(C8-B8)*Inputs!$B$74</f>
+        <f aca="false">-(C8-B8)*Inputs!$B$77</f>
         <v>-45</v>
       </c>
       <c r="D25" s="31" t="n">
-        <f aca="false">-(D8-C8)*Inputs!$B$74</f>
+        <f aca="false">-(D8-C8)*Inputs!$B$77</f>
         <v>-95.94414893617</v>
       </c>
       <c r="E25" s="31" t="n">
-        <f aca="false">-(E8-D8)*Inputs!$B$74</f>
+        <f aca="false">-(E8-D8)*Inputs!$B$77</f>
         <v>-62.2736037234041</v>
       </c>
       <c r="F25" s="31" t="n">
-        <f aca="false">-(F8-E8)*Inputs!$B$74</f>
+        <f aca="false">-(F8-E8)*Inputs!$B$77</f>
         <v>-63.8304438164894</v>
       </c>
       <c r="G25" s="31" t="n">
-        <f aca="false">-(G8-F8)*Inputs!$B$74</f>
+        <f aca="false">-(G8-F8)*Inputs!$B$77</f>
         <v>-65.4262049119017</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="B26" s="34"/>
       <c r="C26" s="31" t="n">
-        <f aca="false">-Inputs!$B$56</f>
+        <f aca="false">-Inputs!$B$59</f>
         <v>-250</v>
       </c>
       <c r="D26" s="31" t="n">
-        <f aca="false">-Inputs!$B$56*0.5</f>
+        <f aca="false">-Inputs!$B$59*0.5</f>
         <v>-125</v>
       </c>
       <c r="E26" s="31" t="n">
@@ -4768,12 +4828,12 @@
         <v>0</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="B27" s="33" t="n">
         <f aca="false">B22+B23+B24+IF(ISNUMBER(B25),B25,0)+IF(ISNUMBER(B26),B26,0)</f>
@@ -4802,7 +4862,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="B28" s="35" t="n">
         <f aca="false">B27/B8</f>
@@ -4831,7 +4891,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="27" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="B29" s="28"/>
       <c r="C29" s="28"/>
@@ -4843,27 +4903,27 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="B30" s="34"/>
       <c r="C30" s="31" t="n">
-        <f aca="false">C27-Inputs!$B$54*(1-Inputs!$B$75)</f>
+        <f aca="false">C27-Inputs!$B$57*(1-Inputs!$B$78)</f>
         <v>303.4</v>
       </c>
       <c r="D30" s="31" t="n">
-        <f aca="false">D27-Inputs!$B$54*(1-Inputs!$B$75)</f>
+        <f aca="false">D27-Inputs!$B$57*(1-Inputs!$B$78)</f>
         <v>1219.3720212766</v>
       </c>
       <c r="E30" s="34"/>
       <c r="F30" s="34"/>
       <c r="G30" s="34"/>
       <c r="H30" s="7" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="B31" s="31" t="n">
         <f aca="false">-Inputs!$B$9*Inputs!$B$8</f>
@@ -4890,15 +4950,15 @@
         <v>-979.575</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="B32" s="30" t="n">
-        <f aca="false">Inputs!$B$43</f>
+        <f aca="false">Inputs!$B$46</f>
         <v>-159</v>
       </c>
       <c r="C32" s="34"/>
@@ -4907,12 +4967,12 @@
       <c r="F32" s="34"/>
       <c r="G32" s="34"/>
       <c r="H32" s="7" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="B33" s="34"/>
       <c r="C33" s="37" t="n">
@@ -4953,17 +5013,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -4974,7 +5034,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="B5" s="38" t="n">
         <f aca="false">Inputs!$B$7*Inputs!$B$8</f>
@@ -4983,7 +5043,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="B6" s="38" t="n">
         <f aca="false">Inputs!$B$15-Inputs!$B$16</f>
@@ -4992,19 +5052,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="B7" s="38" t="n">
-        <f aca="false">Inputs!$B$36</f>
-        <v>626</v>
+        <f aca="false">Inputs!$B$39</f>
+        <v>957.48</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="B8" s="39" t="n">
         <f aca="false">B5/(B5+B6)</f>
@@ -5013,7 +5073,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="B9" s="39" t="n">
         <f aca="false">1-B8</f>
@@ -5022,37 +5082,37 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="B10" s="40" t="n">
-        <f aca="false">Inputs!$B$78+Inputs!$B$79*Inputs!$B$80</f>
+        <f aca="false">Inputs!$B$81+Inputs!$B$82*Inputs!$B$83</f>
         <v>0.0895</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="B11" s="40" t="n">
-        <f aca="false">Inputs!$B$81*(1-Inputs!$B$75)</f>
+        <f aca="false">Inputs!$B$84*(1-Inputs!$B$78)</f>
         <v>0.0418</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="B12" s="41" t="n">
         <f aca="false">B8*B10+B9*B11</f>
         <v>0.0735762453312365</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -5063,24 +5123,24 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="E15" s="26" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="B16" s="38" t="n">
         <f aca="false">Model!D27</f>
@@ -5101,7 +5161,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="B17" s="42" t="n">
         <v>0.7</v>
@@ -5116,12 +5176,12 @@
         <v>3.7</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
       <c r="B18" s="43" t="n">
         <f aca="false">1/(1+B12)^B17</f>
@@ -5142,7 +5202,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="B19" s="44" t="n">
         <f aca="false">B16*B18</f>
@@ -5163,7 +5223,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
@@ -5174,40 +5234,40 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="B22" s="19" t="n">
-        <f aca="false">E16*(1+Inputs!$B$82)/(B12-Inputs!$B$82)</f>
+        <f aca="false">E16*(1+Inputs!$B$85)/(B12-Inputs!$B$85)</f>
         <v>31960.0871104651</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="B23" s="19" t="n">
-        <f aca="false">Model!G14*Inputs!$B$83</f>
+        <f aca="false">Model!G14*Inputs!$B$86</f>
         <v>31291.8569473737</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="B24" s="45" t="n">
         <f aca="false">B22/Model!G14</f>
         <v>8.17083809739135</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="B25" s="39" t="n">
         <f aca="false">(B23*B12-E16)/(B23+E16)</f>
@@ -5216,7 +5276,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="B26" s="46" t="n">
         <f aca="false">AVERAGE(B22,B23)</f>
@@ -5225,7 +5285,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="B27" s="19" t="n">
         <f aca="false">B26*E18</f>
@@ -5234,7 +5294,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
@@ -5245,7 +5305,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
       <c r="B30" s="19" t="n">
         <f aca="false">SUM(B19:E19)</f>
@@ -5254,7 +5314,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
       <c r="B31" s="46" t="n">
         <f aca="false">B30+B27</f>
@@ -5263,46 +5323,46 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
       <c r="B32" s="39" t="n">
         <f aca="false">B27/B31</f>
         <v>0.816013111760449</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
       <c r="B33" s="46" t="n">
         <f aca="false">B31-B6-B7</f>
-        <v>20686.3470252726</v>
+        <v>20354.8670252726</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="B34" s="47" t="n">
         <f aca="false">B33/Inputs!$B$8</f>
-        <v>39.0676997644431</v>
+        <v>38.4416752129794</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="B35" s="39" t="n">
         <f aca="false">B34/Inputs!$B$7-1</f>
-        <v>0.220865617638845</v>
+        <v>0.201302350405606</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="B36" s="45" t="n">
         <f aca="false">B31/Model!D14</f>
@@ -5311,7 +5371,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
       <c r="B37" s="45" t="n">
         <f aca="false">(B5+B6)/Model!D14</f>
@@ -5320,14 +5380,14 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="B38" s="45" t="n">
         <f aca="false">(B5+B6)/Model!C14</f>
         <v>7.70757575757576</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
     </row>
   </sheetData>
@@ -5356,34 +5416,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>0.25</v>
@@ -5395,12 +5455,12 @@
         <v>0.8</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
       <c r="B6" s="21" t="n">
         <v>-0.02</v>
@@ -5412,12 +5472,12 @@
         <v>0.03</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>200</v>
@@ -5429,12 +5489,12 @@
         <v>450</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>350</v>
@@ -5446,12 +5506,12 @@
         <v>200</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>0</v>
@@ -5463,12 +5523,12 @@
         <v>300</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
       <c r="B10" s="21" t="n">
         <v>0.13</v>
@@ -5480,12 +5540,12 @@
         <v>0.2</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
       <c r="B11" s="21" t="n">
         <v>0.09</v>
@@ -5497,12 +5557,12 @@
         <v>0.13</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="B12" s="21" t="n">
         <v>0.075</v>
@@ -5514,12 +5574,12 @@
         <v>0.06</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="B13" s="21" t="n">
         <f aca="false">DCF!B12+0.005</f>
@@ -5534,12 +5594,12 @@
         <v>0.0685762453312365</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="B14" s="23" t="n">
         <v>7</v>
@@ -5551,12 +5611,12 @@
         <v>9.5</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="27" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="B16" s="29"/>
       <c r="C16" s="29"/>
@@ -5565,58 +5625,58 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="B17" s="19" t="n">
-        <f aca="false">Model!C6*(1+B6)+B5*Inputs!$B$59*Inputs!$B$60-Inputs!$B$61</f>
+        <f aca="false">Model!C6*(1+B6)+B5*Inputs!$B$62*Inputs!$B$63-Inputs!$B$64</f>
         <v>15188.9893617021</v>
       </c>
       <c r="C17" s="19" t="n">
-        <f aca="false">Model!C6*(1+C6)+C5*Inputs!$B$59*Inputs!$B$60-Inputs!$B$61</f>
+        <f aca="false">Model!C6*(1+C6)+C5*Inputs!$B$62*Inputs!$B$63-Inputs!$B$64</f>
         <v>16030.1063829787</v>
       </c>
       <c r="D17" s="19" t="n">
-        <f aca="false">Model!C6*(1+D6)+D5*Inputs!$B$59*Inputs!$B$60-Inputs!$B$61</f>
+        <f aca="false">Model!C6*(1+D6)+D5*Inputs!$B$62*Inputs!$B$63-Inputs!$B$64</f>
         <v>16794.8510638298</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="B18" s="19" t="n">
-        <f aca="false">Model!C7*(1+Inputs!$B$70)</f>
+        <f aca="false">Model!C7*(1+Inputs!$B$73)</f>
         <v>8879.33510638298</v>
       </c>
       <c r="C18" s="19" t="n">
-        <f aca="false">Model!C7*(1+Inputs!$B$70)</f>
+        <f aca="false">Model!C7*(1+Inputs!$B$73)</f>
         <v>8879.33510638298</v>
       </c>
       <c r="D18" s="19" t="n">
-        <f aca="false">Model!C7*(1+Inputs!$B$70)</f>
+        <f aca="false">Model!C7*(1+Inputs!$B$73)</f>
         <v>8879.33510638298</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="B19" s="19" t="n">
-        <f aca="false">Model!C11+(B5*Inputs!$B$59*Inputs!$B$60-Inputs!$B$61)+Model!C6*B6*Inputs!$B$64+(B7-B8)*Model!C6/Model!C8</f>
+        <f aca="false">Model!C11+(B5*Inputs!$B$62*Inputs!$B$63-Inputs!$B$64)+Model!C6*B6*Inputs!$B$67+(B7-B8)*Model!C6/Model!C8</f>
         <v>2445.03191489362</v>
       </c>
       <c r="C19" s="19" t="n">
-        <f aca="false">Model!C11+(C5*Inputs!$B$59*Inputs!$B$60-Inputs!$B$61)+Model!C6*C6*Inputs!$B$64+(C7-C8)*Model!C6/Model!C8</f>
+        <f aca="false">Model!C11+(C5*Inputs!$B$62*Inputs!$B$63-Inputs!$B$64)+Model!C6*C6*Inputs!$B$67+(C7-C8)*Model!C6/Model!C8</f>
         <v>3092.77659574468</v>
       </c>
       <c r="D19" s="19" t="n">
-        <f aca="false">Model!C11+(D5*Inputs!$B$59*Inputs!$B$60-Inputs!$B$61)+Model!C6*D6*Inputs!$B$64+(D7-D8)*Model!C6/Model!C8</f>
+        <f aca="false">Model!C11+(D5*Inputs!$B$62*Inputs!$B$63-Inputs!$B$64)+Model!C6*D6*Inputs!$B$67+(D7-D8)*Model!C6/Model!C8</f>
         <v>3771.15957446809</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="B20" s="19" t="n">
         <f aca="false">Model!C12+B9+(B7-B8)*Model!C7/Model!C8</f>
@@ -5633,7 +5693,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="B21" s="46" t="n">
         <f aca="false">B19+B20+Model!C13</f>
@@ -5650,81 +5710,81 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="B22" s="19" t="n">
-        <f aca="false">(B17+B18)*(1+Inputs!$B$70)^3</f>
+        <f aca="false">(B17+B18)*(1+Inputs!$B$73)^3</f>
         <v>25918.952979139</v>
       </c>
       <c r="C22" s="19" t="n">
-        <f aca="false">(C17+C18)*(1+Inputs!$B$70)^3</f>
+        <f aca="false">(C17+C18)*(1+Inputs!$B$73)^3</f>
         <v>26824.7440138796</v>
       </c>
       <c r="D22" s="19" t="n">
-        <f aca="false">(D17+D18)*(1+Inputs!$B$70)^3</f>
+        <f aca="false">(D17+D18)*(1+Inputs!$B$73)^3</f>
         <v>27648.2903912068</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="B23" s="46" t="n">
-        <f aca="false">B17*(1+Inputs!$B$70)^3*B10+B18*(1+Inputs!$B$70)^3*B11+Model!C13</f>
+        <f aca="false">B17*(1+Inputs!$B$73)^3*B10+B18*(1+Inputs!$B$73)^3*B11+Model!C13</f>
         <v>2911.98097799618</v>
       </c>
       <c r="C23" s="46" t="n">
-        <f aca="false">C17*(1+Inputs!$B$70)^3*C10+C18*(1+Inputs!$B$70)^3*C11+Model!C13</f>
+        <f aca="false">C17*(1+Inputs!$B$73)^3*C10+C18*(1+Inputs!$B$73)^3*C11+Model!C13</f>
         <v>3911.48211842171</v>
       </c>
       <c r="D23" s="46" t="n">
-        <f aca="false">D17*(1+Inputs!$B$70)^3*D10+D18*(1+Inputs!$B$70)^3*D11+Model!C13</f>
+        <f aca="false">D17*(1+Inputs!$B$73)^3*D10+D18*(1+Inputs!$B$73)^3*D11+Model!C13</f>
         <v>4785.31298698055</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="B24" s="19" t="n">
-        <f aca="false">(B23-B22*Inputs!$B$73)*(1-Inputs!$B$75)+B22*Inputs!$B$73-B22*B12-B22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74</f>
+        <f aca="false">(B23-B22*Inputs!$B$76)*(1-Inputs!$B$78)+B22*Inputs!$B$76-B22*B12-B22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77</f>
         <v>703.611008555435</v>
       </c>
       <c r="C24" s="19" t="n">
-        <f aca="false">(C23-C22*Inputs!$B$73)*(1-Inputs!$B$75)+C22*Inputs!$B$73-C22*C12-C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74</f>
+        <f aca="false">(C23-C22*Inputs!$B$76)*(1-Inputs!$B$78)+C22*Inputs!$B$76-C22*C12-C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77</f>
         <v>1678.72692925291</v>
       </c>
       <c r="D24" s="19" t="n">
-        <f aca="false">(D23-D22*Inputs!$B$73)*(1-Inputs!$B$75)+D22*Inputs!$B$73-D22*D12-D22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74</f>
+        <f aca="false">(D23-D22*Inputs!$B$76)*(1-Inputs!$B$78)+D22*Inputs!$B$76-D22*D12-D22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77</f>
         <v>2441.35276753128</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="B25" s="19" t="n">
-        <f aca="false">(B21-(B17+B18)*Inputs!$B$73)*(1-Inputs!$B$75)+(B17+B18)*Inputs!$B$73-Inputs!$B$71-Inputs!$B$56*0.5</f>
+        <f aca="false">(B21-(B17+B18)*Inputs!$B$76)*(1-Inputs!$B$78)+(B17+B18)*Inputs!$B$76-Inputs!$B$74-Inputs!$B$59*0.5</f>
         <v>919.102042553192</v>
       </c>
       <c r="C25" s="19" t="n">
-        <f aca="false">(C21-(C17+C18)*Inputs!$B$73)*(1-Inputs!$B$75)+(C17+C18)*Inputs!$B$73-Inputs!$B$71-Inputs!$B$56*0.5</f>
+        <f aca="false">(C21-(C17+C18)*Inputs!$B$76)*(1-Inputs!$B$78)+(C17+C18)*Inputs!$B$76-Inputs!$B$74-Inputs!$B$59*0.5</f>
         <v>1596.51617021277</v>
       </c>
       <c r="D25" s="19" t="n">
-        <f aca="false">(D21-(D17+D18)*Inputs!$B$73)*(1-Inputs!$B$75)+(D17+D18)*Inputs!$B$73-Inputs!$B$71-Inputs!$B$56*0.5</f>
+        <f aca="false">(D21-(D17+D18)*Inputs!$B$76)*(1-Inputs!$B$78)+(D17+D18)*Inputs!$B$76-Inputs!$B$74-Inputs!$B$59*0.5</f>
         <v>2295.74905531915</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="B26" s="19" t="n">
         <f aca="false">B25/(1+B13)^0.7+(B25*2/3+B24/3)/(1+B13)^1.7+(B25/3+B24*2/3)/(1+B13)^2.7+B24/(1+B13)^3.7</f>
@@ -5739,29 +5799,29 @@
         <v>8196.46184115283</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="B27" s="19" t="n">
-        <f aca="false">AVERAGE(B24*(1+Inputs!$B$82)/(B13-Inputs!$B$82),B23*B14)</f>
+        <f aca="false">AVERAGE(B24*(1+Inputs!$B$85)/(B13-Inputs!$B$85),B23*B14)</f>
         <v>16317.9937796055</v>
       </c>
       <c r="C27" s="19" t="n">
-        <f aca="false">AVERAGE(C24*(1+Inputs!$B$82)/(C13-Inputs!$B$82),C23*C14)</f>
+        <f aca="false">AVERAGE(C24*(1+Inputs!$B$85)/(C13-Inputs!$B$85),C23*C14)</f>
         <v>31625.9720289194</v>
       </c>
       <c r="D27" s="19" t="n">
-        <f aca="false">AVERAGE(D24*(1+Inputs!$B$82)/(D13-Inputs!$B$82),D23*D14)</f>
+        <f aca="false">AVERAGE(D24*(1+Inputs!$B$85)/(D13-Inputs!$B$85),D23*D14)</f>
         <v>48361.8988915826</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
       <c r="B28" s="46" t="n">
         <f aca="false">B26+B27/(1+B13)^3.7</f>
@@ -5778,58 +5838,58 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="B29" s="19" t="n">
         <f aca="false">B28-DCF!B6-DCF!B7</f>
-        <v>5998.19323666879</v>
+        <v>5666.71323666879</v>
       </c>
       <c r="C29" s="19" t="n">
         <f aca="false">C28-DCF!B6-DCF!B7</f>
-        <v>20815.5184068871</v>
+        <v>20484.0384068871</v>
       </c>
       <c r="D29" s="19" t="n">
         <f aca="false">D28-DCF!B6-DCF!B7</f>
-        <v>36917.0057030091</v>
+        <v>36585.5257030091</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="B30" s="47" t="n">
         <f aca="false">B29/Inputs!$B$8</f>
-        <v>11.3280325527267</v>
+        <v>10.7020080012631</v>
       </c>
       <c r="C30" s="47" t="n">
         <f aca="false">C29/Inputs!$B$8</f>
-        <v>39.311649493649</v>
+        <v>38.6856249421854</v>
       </c>
       <c r="D30" s="47" t="n">
         <f aca="false">D29/Inputs!$B$8</f>
-        <v>69.7205017998283</v>
+        <v>69.0944772483647</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
       <c r="B31" s="39" t="n">
         <f aca="false">B30/Inputs!$B$7-1</f>
-        <v>-0.64599898272729</v>
+        <v>-0.665562249960529</v>
       </c>
       <c r="C31" s="39" t="n">
         <f aca="false">C30/Inputs!$B$7-1</f>
-        <v>0.228489046676531</v>
+        <v>0.208925779443292</v>
       </c>
       <c r="D31" s="39" t="n">
         <f aca="false">D30/Inputs!$B$7-1</f>
-        <v>1.17876568124464</v>
+        <v>1.1592024140114</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="B32" s="39" t="n">
         <f aca="false">B27/(1+B13)^3.7/B28</f>
@@ -5846,7 +5906,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
       <c r="B33" s="45" t="n">
         <f aca="false">B28/B21</f>
@@ -5863,7 +5923,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="B35" s="21" t="n">
         <v>0.3</v>
@@ -5877,14 +5937,14 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
       <c r="B36" s="47" t="n">
         <f aca="false">SUMPRODUCT(B30:D30,B35:D35)/SUM(B35:D35)</f>
-        <v>38.5187774879172</v>
+        <v>37.8927529364535</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
     </row>
   </sheetData>
@@ -5912,17 +5972,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5950,28 +6010,28 @@
         <v>0.13</v>
       </c>
       <c r="B6" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*B$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>22.9367338935485</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*B$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>22.3107093420848</v>
       </c>
       <c r="C6" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*C$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>25.2756235011637</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*C$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>24.6495989497001</v>
       </c>
       <c r="D6" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*D$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>27.6145131087789</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*D$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>26.9884885573153</v>
       </c>
       <c r="E6" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*E$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>29.9534027163942</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*E$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>29.3273781649305</v>
       </c>
       <c r="F6" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*F$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>33.461737127817</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*F$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>32.8357125763534</v>
       </c>
       <c r="G6" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A6+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*G$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>35.8006267354323</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A6+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*G$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>35.1746021839686</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5979,28 +6039,28 @@
         <v>0.15</v>
       </c>
       <c r="B7" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*B$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>28.9939692954878</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*B$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>28.3679447440242</v>
       </c>
       <c r="C7" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*C$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>31.5835623647027</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*C$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>30.9575378132391</v>
       </c>
       <c r="D7" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*D$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>34.1731554339176</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*D$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>33.5471308824539</v>
       </c>
       <c r="E7" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*E$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>36.7627485031325</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*E$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>36.1367239516688</v>
       </c>
       <c r="F7" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*F$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>40.6471381069548</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*F$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>40.0211135554911</v>
       </c>
       <c r="G7" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A7+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*G$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>43.2367311761696</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A7+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*G$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>42.610706624706</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6008,28 +6068,28 @@
         <v>0.17</v>
       </c>
       <c r="B8" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*B$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>35.0512046974272</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*B$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>34.4251801459636</v>
       </c>
       <c r="C8" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*C$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>37.8915012282417</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*C$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>37.2654766767781</v>
       </c>
       <c r="D8" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*D$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>40.7317977590563</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*D$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>40.1057732075926</v>
       </c>
       <c r="E8" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*E$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>43.5720942898708</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*E$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>42.9460697384071</v>
       </c>
       <c r="F8" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*F$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>47.8325390860925</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*F$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>47.2065145346289</v>
       </c>
       <c r="G8" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A8+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*G$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>50.6728356169071</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A8+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*G$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>50.0468110654434</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6037,28 +6097,28 @@
         <v>0.19</v>
       </c>
       <c r="B9" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*B$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>41.1084400993666</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*B$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>40.482415547903</v>
       </c>
       <c r="C9" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*C$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>44.1994400917808</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*C$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>43.5734155403171</v>
       </c>
       <c r="D9" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*D$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>47.2904400841949</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*D$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>46.6644155327313</v>
       </c>
       <c r="E9" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*E$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>50.3814400766091</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*E$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>49.7554155251454</v>
       </c>
       <c r="F9" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*F$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>55.0179400652303</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*F$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>54.3919155137666</v>
       </c>
       <c r="G9" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A9+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*G$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>58.1089400576444</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A9+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*G$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>57.4829155061808</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6066,55 +6126,55 @@
         <v>0.21</v>
       </c>
       <c r="B10" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*B$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>47.165675501306</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*B$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>46.5396509498424</v>
       </c>
       <c r="C10" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*C$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>50.5073789553198</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*C$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>49.8813544038562</v>
       </c>
       <c r="D10" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*D$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>53.8490824093336</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*D$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>53.2230578578699</v>
       </c>
       <c r="E10" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*E$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>57.1907858633473</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*E$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>56.5647613118837</v>
       </c>
       <c r="F10" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*F$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>62.203341044368</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*F$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>61.5773164929044</v>
       </c>
       <c r="G10" s="50" t="n">
-        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$73)*(1-Inputs!$B$75)+Scenarios!C22*Inputs!$B$73-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$70/(1+Inputs!$B$70)*Inputs!$B$74)*(1+Inputs!$B$82)/(Scenarios!C13-Inputs!$B$82),(Scenarios!C17*(1+Inputs!$B$70)^3*$A10+Scenarios!C18*(1+Inputs!$B$70)^3*Scenarios!C11+Model!C13)*G$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
-        <v>65.5450444983818</v>
+        <f aca="false">((Scenarios!C25/(1+Scenarios!C13)^0.7+(Scenarios!C25*2/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/3)/(1+Scenarios!C13)^1.7+(Scenarios!C25/3+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*2/3)/(1+Scenarios!C13)^2.7+(((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)/(1+Scenarios!C13)^3.7)+AVERAGE((((Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)-Scenarios!C22*Inputs!$B$76)*(1-Inputs!$B$78)+Scenarios!C22*Inputs!$B$76-Scenarios!C22*Scenarios!C12-Scenarios!C22*Inputs!$B$73/(1+Inputs!$B$73)*Inputs!$B$77)*(1+Inputs!$B$85)/(Scenarios!C13-Inputs!$B$85),(Scenarios!C17*(1+Inputs!$B$73)^3*$A10+Scenarios!C18*(1+Inputs!$B$73)^3*Scenarios!C11+Model!C13)*G$5)/(1+Scenarios!C13)^3.7-DCF!B6-DCF!B7)/Inputs!$B$8</f>
+        <v>64.9190199469181</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6122,15 +6182,15 @@
         <v>0</v>
       </c>
       <c r="B16" s="44" t="n">
-        <f aca="false">A16*Inputs!$B$59</f>
+        <f aca="false">A16*Inputs!$B$62</f>
         <v>0</v>
       </c>
       <c r="C16" s="44" t="n">
-        <f aca="false">Scenarios!C21-(Scenarios!C5-A16)*Inputs!$B$59*Inputs!$B$60</f>
+        <f aca="false">Scenarios!C21-(Scenarios!C5-A16)*Inputs!$B$62*Inputs!$B$63</f>
         <v>3370.86170212766</v>
       </c>
       <c r="D16" s="51" t="n">
-        <f aca="false">C16/((Inputs!$B$47+Inputs!$B$48)/2)-1</f>
+        <f aca="false">C16/((Inputs!$B$50+Inputs!$B$51)/2)-1</f>
         <v>0.0214732430689877</v>
       </c>
       <c r="E16" s="52" t="n">
@@ -6143,15 +6203,15 @@
         <v>0.25</v>
       </c>
       <c r="B17" s="44" t="n">
-        <f aca="false">A17*Inputs!$B$59</f>
+        <f aca="false">A17*Inputs!$B$62</f>
         <v>42.5</v>
       </c>
       <c r="C17" s="44" t="n">
-        <f aca="false">Scenarios!C21-(Scenarios!C5-A17)*Inputs!$B$59*Inputs!$B$60</f>
+        <f aca="false">Scenarios!C21-(Scenarios!C5-A17)*Inputs!$B$62*Inputs!$B$63</f>
         <v>3753.36170212766</v>
       </c>
       <c r="D17" s="51" t="n">
-        <f aca="false">C17/((Inputs!$B$47+Inputs!$B$48)/2)-1</f>
+        <f aca="false">C17/((Inputs!$B$50+Inputs!$B$51)/2)-1</f>
         <v>0.137382333978079</v>
       </c>
       <c r="E17" s="52" t="n">
@@ -6164,15 +6224,15 @@
         <v>0.5</v>
       </c>
       <c r="B18" s="44" t="n">
-        <f aca="false">A18*Inputs!$B$59</f>
+        <f aca="false">A18*Inputs!$B$62</f>
         <v>85</v>
       </c>
       <c r="C18" s="44" t="n">
-        <f aca="false">Scenarios!C21-(Scenarios!C5-A18)*Inputs!$B$59*Inputs!$B$60</f>
+        <f aca="false">Scenarios!C21-(Scenarios!C5-A18)*Inputs!$B$62*Inputs!$B$63</f>
         <v>4135.86170212766</v>
       </c>
       <c r="D18" s="51" t="n">
-        <f aca="false">C18/((Inputs!$B$47+Inputs!$B$48)/2)-1</f>
+        <f aca="false">C18/((Inputs!$B$50+Inputs!$B$51)/2)-1</f>
         <v>0.25329142488717</v>
       </c>
       <c r="E18" s="52" t="n">
@@ -6185,15 +6245,15 @@
         <v>0.75</v>
       </c>
       <c r="B19" s="44" t="n">
-        <f aca="false">A19*Inputs!$B$59</f>
+        <f aca="false">A19*Inputs!$B$62</f>
         <v>127.5</v>
       </c>
       <c r="C19" s="44" t="n">
-        <f aca="false">Scenarios!C21-(Scenarios!C5-A19)*Inputs!$B$59*Inputs!$B$60</f>
+        <f aca="false">Scenarios!C21-(Scenarios!C5-A19)*Inputs!$B$62*Inputs!$B$63</f>
         <v>4518.36170212766</v>
       </c>
       <c r="D19" s="51" t="n">
-        <f aca="false">C19/((Inputs!$B$47+Inputs!$B$48)/2)-1</f>
+        <f aca="false">C19/((Inputs!$B$50+Inputs!$B$51)/2)-1</f>
         <v>0.369200515796261</v>
       </c>
       <c r="E19" s="52" t="n">
@@ -6206,15 +6266,15 @@
         <v>1</v>
       </c>
       <c r="B20" s="44" t="n">
-        <f aca="false">A20*Inputs!$B$59</f>
+        <f aca="false">A20*Inputs!$B$62</f>
         <v>170</v>
       </c>
       <c r="C20" s="44" t="n">
-        <f aca="false">Scenarios!C21-(Scenarios!C5-A20)*Inputs!$B$59*Inputs!$B$60</f>
+        <f aca="false">Scenarios!C21-(Scenarios!C5-A20)*Inputs!$B$62*Inputs!$B$63</f>
         <v>4900.86170212766</v>
       </c>
       <c r="D20" s="51" t="n">
-        <f aca="false">C20/((Inputs!$B$47+Inputs!$B$48)/2)-1</f>
+        <f aca="false">C20/((Inputs!$B$50+Inputs!$B$51)/2)-1</f>
         <v>0.485109606705351</v>
       </c>
       <c r="E20" s="52" t="n">
@@ -6224,7 +6284,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
     </row>
   </sheetData>
@@ -6253,12 +6313,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -6267,10 +6327,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>28</v>
@@ -6278,33 +6338,33 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="B5" s="53" t="n">
-        <f aca="false">Inputs!$B$86</f>
+        <f aca="false">Inputs!$B$89</f>
         <v>12.2</v>
       </c>
       <c r="C5" s="40" t="n">
-        <f aca="false">Inputs!$B$87</f>
+        <f aca="false">Inputs!$B$90</f>
         <v>0.21</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="B6" s="53" t="n">
-        <f aca="false">Inputs!$B$88</f>
+        <f aca="false">Inputs!$B$91</f>
         <v>7.2</v>
       </c>
       <c r="C6" s="40" t="n">
-        <f aca="false">Inputs!$B$89</f>
+        <f aca="false">Inputs!$B$92</f>
         <v>0.15</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="B7" s="52" t="n">
         <f aca="false">DCF!B38</f>
@@ -6317,7 +6377,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="C8" s="51" t="n">
         <f aca="false">Model!C16</f>
@@ -6326,7 +6386,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -6335,24 +6395,24 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>184</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="B12" s="44" t="n">
         <f aca="false">Model!E11</f>
@@ -6366,12 +6426,12 @@
         <v>25139.2143351064</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="B13" s="44" t="n">
         <f aca="false">Model!E12</f>
@@ -6385,12 +6445,12 @@
         <v>6507.44271609042</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="B14" s="44" t="n">
         <f aca="false">Model!E13</f>
@@ -6407,7 +6467,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="D15" s="46" t="n">
         <f aca="false">SUM(D12:D14)</f>
@@ -6416,62 +6476,62 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="D16" s="44" t="n">
         <f aca="false">-DCF!B6-DCF!B7</f>
-        <v>-9117</v>
+        <v>-9448.48</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="D17" s="44" t="n">
-        <f aca="false">-Inputs!$B$56*1.5</f>
+        <f aca="false">-Inputs!$B$59*1.5</f>
         <v>-375</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="D18" s="46" t="n">
         <f aca="false">D15+D16+D17</f>
-        <v>21479.6570511968</v>
+        <v>21148.1770511968</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="D19" s="47" t="n">
         <f aca="false">D18/Inputs!$B$8</f>
-        <v>40.5659245537239</v>
+        <v>39.9399000022603</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
       <c r="D20" s="51" t="n">
         <f aca="false">D19/Inputs!$B$7-1</f>
-        <v>0.267685142303872</v>
+        <v>0.248121875070633</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="D22" s="52" t="n">
         <f aca="false">((DCF!B5-D17-D16)-D12-D14)/B13</f>
-        <v>1.96953048700958</v>
+        <v>2.30063136549637</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
     </row>
   </sheetData>

</xml_diff>